<commit_message>
feat: battle bar limit of 70
battle bar limit of 70, no repeated values in line 1, party skill box,
Arcane Shield rate

Line 1 of a skill no longer repeats the values the box below shows
(setting line1_values). Line 1 of techniques and spells and the joint
skill sentences fit the 70 characters the battle bar draws; 44 skill and
22 joint sentences reworded in the rules workbook. Party skill lines fit
their box (50). Arcane Shield states the activation rate the DT2-2 wiki
measured, marked as a guide figure.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_joint_skill_text.xlsx
+++ b/mod_project/data_tables/qol_joint_skill_text.xlsx
@@ -834,11 +834,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Deal non-elemental damage to all enemies. 100% chance of causing sleep.</t>
+          <t>Deal non-elemental damage to all enemies. 100% chance of sleep.</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="F8" t="n">
         <v>3</v>
@@ -940,11 +940,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Deal non-elemental damage and lower DEF and magic defense (-20%) for all enemies.</t>
+          <t>Non-elemental damage to all enemies. DEF and magic defense -20%.</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="F10" t="n">
         <v>3</v>
@@ -1046,11 +1046,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Activate Circle Brave (+16%), Circle Protect (+16%) and Moon Curtain (+25%) at once.</t>
+          <t>Circle Brave (+16%), Circle Protect (+16%) and Moon Curtain (+25%).</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="F12" t="n">
         <v>3</v>
@@ -1152,11 +1152,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Deal damage with an 85% chance to silence/freeze. Pierces to the back row.</t>
+          <t>Deal damage through to the back row. 85% chance to silence/freeze.</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="F14" t="n">
         <v>3</v>
@@ -1205,11 +1205,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Form up to increase speed (+50%) and physical accuracy (+75%) for all allies.</t>
+          <t>Form up: speed +50% and physical accuracy +75% for all allies.</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="F15" t="n">
         <v>3</v>
@@ -1417,11 +1417,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Deal damage and reduce physical attack/defense (-25%). Pierces to the back row.</t>
+          <t>Deal damage through to the back row. Physical attack/defense -25%.</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="F19" t="n">
         <v>3</v>
@@ -1629,11 +1629,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Deal physical damage, with a 90% chance to delay the target's next turn.</t>
+          <t>Deal physical damage. 90% chance to delay the target's next turn.</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F23" t="n">
         <v>3</v>
@@ -1735,11 +1735,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Deal physical damage to one enemy. 100% chance of poison/paralysis/sleep.</t>
+          <t>Physical damage to one enemy. 100% chance of poison/paralysis/sleep.</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F25" t="n">
         <v>3</v>
@@ -2212,11 +2212,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Waste one enemy and poison the target (100%) with a rare gun-type weapon.</t>
+          <t>Waste one enemy and poison it (100%) with a rare gun.</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="F34" t="n">
         <v>2</v>
@@ -2265,11 +2265,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Cancel all enemy chants, dances, songs, and dolls with a superior performance.</t>
+          <t>Cancel enemy chants, dances, songs and dolls by outperforming them.</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="F35" t="n">
         <v>3</v>
@@ -2371,11 +2371,11 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Slice a random enemy 2-5 times with the power of friendship. And swords.</t>
+          <t>Slice a random enemy 2-5 times with friendship power. And swords.</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F37" t="n">
         <v>3</v>
@@ -2424,11 +2424,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Rough up (4 hits) and poison (100%) one enemy with the power of darkness.</t>
+          <t>Rough up (4 hits) and poison (100%) one enemy with dark power.</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="F38" t="n">
         <v>3</v>
@@ -2530,11 +2530,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Fire two arrows of light that pierce to the back row and may silence (50%).</t>
+          <t>Two arrows of light pierce to the back row and may silence (50%).</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F40" t="n">
         <v>3</v>
@@ -2583,11 +2583,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>The deadly Maid Beam pierces to the back row and begins petrifying targets (75%).</t>
+          <t>The deadly Maid Beam pierces to the back row. Petrifying (75%).</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="F41" t="n">
         <v>3</v>
@@ -2689,11 +2689,11 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Heal the party to full HP and remove debuffs and ailments with a secret potion.</t>
+          <t>A secret potion: full HP for the party, debuffs and ailments removed.</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="F43" t="n">
         <v>3</v>
@@ -2795,11 +2795,11 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Hurl 5% of your wallet at one enemy for up to 10000 damage. (You won't get it back.)</t>
+          <t>Hurl 5% of your wallet at one enemy (max 10000 damage). No refunds.</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="F45" t="n">
         <v>4</v>
@@ -2848,11 +2848,11 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Dish out paralysis (50%) and 7 times the user's level in damage to all enemies.</t>
+          <t>Dish out paralysis (50%) and 7x user level damage to all enemies.</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="F46" t="n">
         <v>4</v>
@@ -2901,11 +2901,11 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Gain 4x the current enemies' value in gold at the end of battle. (Min. 100)</t>
+          <t>Gain 4x the enemies' gold value at the end of battle. (Min. 100)</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="F47" t="n">
         <v>5</v>
@@ -3007,11 +3007,11 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Waste one enemy and lower target's phys. DEF (-35%) with a rare gun-type weapon.</t>
+          <t>Waste one enemy and lower its phys. DEF (-35%) with a rare gun.</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="F49" t="n">
         <v>4</v>
@@ -3113,11 +3113,11 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Deal 77 times the user's level in damage to one enemy. Jokers are wild!</t>
+          <t>Deal 77x the user's level in damage to one enemy. Jokers are wild!</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F51" t="n">
         <v>5</v>
@@ -3166,11 +3166,11 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Deal damage and likely petrify all enemies by tugging their heartstrings.</t>
+          <t>Damage and likely petrify all enemies by tugging their heartstrings.</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F52" t="n">
         <v>3</v>
@@ -3219,11 +3219,11 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>With three firearms in your hands, rain lead upon your enemies at random (9 hits).</t>
+          <t>Three firearms in hand, rain lead on random enemies (9 hits).</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="F53" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
feat: close QoL: resistances without percent sign
close QoL: resistances without percent sign; remove the earlier mixed
build

Resistances are written as the status screen writes them (Fire
resistance +20). The tools and workbooks of the earlier mixed build are
deleted on request. Docs record what the Balance variant inherits.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_joint_skill_text.xlsx
+++ b/mod_project/data_tables/qol_joint_skill_text.xlsx
@@ -1046,11 +1046,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Circle Brave (+16%), Circle Protect (+16%) and Moon Curtain (+25%).</t>
+          <t>Circle Brave (+16%), Circle Protect (+16%) and Moon Curtain (+25).</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F12" t="n">
         <v>3</v>

</xml_diff>